<commit_message>
Test is running correctly
</commit_message>
<xml_diff>
--- a/utils/testdata.xlsx
+++ b/utils/testdata.xlsx
@@ -1,64 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
-  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rfnsh\PycharmProjects\mobileAutomationProject\utils\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tomas\PycharmProjects\AppiumPythonFork\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B0EBB2-8DB0-47D1-8FB6-68332FA7A5DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{466A1274-6B92-43C7-9BD7-72A0CCCEB455}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
-    <t>country</t>
+    <t>email</t>
   </si>
   <si>
-    <t>name</t>
+    <t>password</t>
   </si>
   <si>
-    <t>gender</t>
+    <t>example@bod.com</t>
   </si>
   <si>
-    <t>Bangladesh</t>
-  </si>
-  <si>
-    <t>Faroque</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>Dina</t>
-  </si>
-  <si>
-    <t>Female</t>
+    <t>10203040</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,13 +54,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -97,14 +69,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -113,10 +77,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -285,6 +249,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -311,24 +276,25 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -389,67 +355,43 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89804D22-CEDE-41D6-973D-20FCBB17406E}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="8.777344" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="1" width="18.33203" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.10938" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.777344" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.777344" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -457,11 +399,10 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{3CF3B7EA-7F8A-4040-8684-BB5C9285F586}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25">
       <formula1>"Male, Female"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup r:id="rId1" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added parametrized login tests
</commit_message>
<xml_diff>
--- a/utils/testdata.xlsx
+++ b/utils/testdata.xlsx
@@ -8,10 +8,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="1" r:id="rId1"/>
+    <sheet name="incorrect_login" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr/>
 </workbook>
@@ -30,6 +31,33 @@
   </si>
   <si>
     <t>10203040</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>element</t>
+  </si>
+  <si>
+    <t>Username is required</t>
+  </si>
+  <si>
+    <t>By.ID, "com.saucelabs.mydemoapp.android:id/nameErrorTV"</t>
+  </si>
+  <si>
+    <t>bod@example.com</t>
+  </si>
+  <si>
+    <t>Enter Password</t>
+  </si>
+  <si>
+    <t>By.ID, "com.saucelabs.mydemoapp.android:id/passwordErrorTV"</t>
+  </si>
+  <si>
+    <t>alice@example.com</t>
+  </si>
+  <si>
+    <t>Sorry this user has been locked out.</t>
   </si>
 </sst>
 </file>
@@ -405,4 +433,68 @@
   </dataValidations>
   <pageSetup r:id="rId1" orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.85547" customWidth="1"/>
+    <col min="2" max="2" width="14.71094" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="58.85547" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2">
+        <v>10203040</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>10203040</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>